<commit_message>
functional diversity results with presence/absence data Figures from community analisis updated Summary of community level analysis
</commit_message>
<xml_diff>
--- a/results/FD x microclimatic gradients.xlsx
+++ b/results/FD x microclimatic gradients.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="17310" windowHeight="16590" activeTab="1"/>
+    <workbookView minimized="1" xWindow="0" yWindow="0" windowWidth="17310" windowHeight="16590" firstSheet="1" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="FD vs micro MED" sheetId="2" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="97" uniqueCount="18">
   <si>
     <t>Func.div</t>
   </si>
@@ -67,6 +67,18 @@
   </si>
   <si>
     <t>W.plant.Rao.ab</t>
+  </si>
+  <si>
+    <t>Germ.Mpd.pa</t>
+  </si>
+  <si>
+    <t>Germ.Rao.pa</t>
+  </si>
+  <si>
+    <t>W.plant.Mpd.pa</t>
+  </si>
+  <si>
+    <t>W.plant.Rao.pa</t>
   </si>
 </sst>
 </file>
@@ -110,7 +122,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="5">
     <border>
       <left/>
       <right/>
@@ -133,21 +145,67 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="11" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -428,7 +486,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F17"/>
+  <dimension ref="A1:F37"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="15.28515625" bestFit="1" customWidth="1"/>
@@ -455,307 +513,682 @@
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A2" s="3" t="s">
+      <c r="A2" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="B2" s="4" t="s">
+      <c r="B2" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="C2" s="4">
+      <c r="C2" s="3">
         <v>-1.4330432133352201E-3</v>
       </c>
-      <c r="D2" s="4">
+      <c r="D2" s="3">
         <v>8.3215150382062004E-4</v>
       </c>
-      <c r="E2" s="4">
+      <c r="E2" s="3">
         <v>-1.72209412199071</v>
       </c>
-      <c r="F2" s="4">
+      <c r="F2" s="3">
         <v>9.1920324804300499E-2</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A3" s="3"/>
-      <c r="B3" s="4" t="s">
+      <c r="A3" s="7"/>
+      <c r="B3" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="C3" s="4">
+      <c r="C3" s="3">
         <v>1.2561425206584599E-3</v>
       </c>
-      <c r="D3" s="4">
+      <c r="D3" s="3">
         <v>9.2128794268652304E-4</v>
       </c>
-      <c r="E3" s="4">
+      <c r="E3" s="3">
         <v>1.36346354104612</v>
       </c>
-      <c r="F3" s="4">
+      <c r="F3" s="3">
         <v>0.179519189577838</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A4" s="3"/>
-      <c r="B4" s="4" t="s">
+      <c r="A4" s="7"/>
+      <c r="B4" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="C4" s="5">
+      <c r="C4" s="4">
         <v>2.3018656176016299E-5</v>
       </c>
-      <c r="D4" s="5">
+      <c r="D4" s="4">
         <v>7.28160820464917E-5</v>
       </c>
-      <c r="E4" s="4">
+      <c r="E4" s="3">
         <v>0.31612049878376303</v>
       </c>
-      <c r="F4" s="4">
+      <c r="F4" s="3">
         <v>0.75337271857259103</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A5" s="3"/>
-      <c r="B5" s="6" t="s">
+      <c r="A5" s="7"/>
+      <c r="B5" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="C5" s="4">
+      <c r="C5" s="3">
         <v>1.0623548648650001E-3</v>
       </c>
-      <c r="D5" s="4">
+      <c r="D5" s="3">
         <v>5.3458737070734004E-4</v>
       </c>
-      <c r="E5" s="4">
+      <c r="E5" s="3">
         <v>1.9872427278993501</v>
       </c>
-      <c r="F5" s="6">
+      <c r="F5" s="5">
         <v>5.3002680223302498E-2</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A6" s="3" t="s">
+      <c r="A6" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="B6" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="C6" s="3">
+        <v>-1.0493605744864201E-3</v>
+      </c>
+      <c r="D6" s="3">
+        <v>4.18624134669235E-4</v>
+      </c>
+      <c r="E6" s="3">
+        <v>-2.5066891456593701</v>
+      </c>
+      <c r="F6" s="6">
+        <v>1.5867367626586599E-2</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A7" s="9"/>
+      <c r="B7" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="C7" s="3">
+        <v>8.5904403786840296E-4</v>
+      </c>
+      <c r="D7" s="3">
+        <v>4.6346532574611702E-4</v>
+      </c>
+      <c r="E7" s="3">
+        <v>1.8535238563650001</v>
+      </c>
+      <c r="F7" s="3">
+        <v>7.0370066942847503E-2</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A8" s="9"/>
+      <c r="B8" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="C8" s="4">
+        <v>8.0197993648781099E-5</v>
+      </c>
+      <c r="D8" s="4">
+        <v>3.6631033167353902E-5</v>
+      </c>
+      <c r="E8" s="3">
+        <v>2.1893456644366398</v>
+      </c>
+      <c r="F8" s="6">
+        <v>3.3798841405545003E-2</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A9" s="10"/>
+      <c r="B9" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="C9" s="3">
+        <v>5.2686406238522301E-4</v>
+      </c>
+      <c r="D9" s="3">
+        <v>2.6893080699845999E-4</v>
+      </c>
+      <c r="E9" s="3">
+        <v>1.9591063897273799</v>
+      </c>
+      <c r="F9" s="5">
+        <v>5.6313700229205801E-2</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A10" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="B6" s="7" t="s">
+      <c r="B10" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="C6" s="4">
+      <c r="C10" s="3">
         <v>-1.94466440063176E-3</v>
       </c>
-      <c r="D6" s="4">
+      <c r="D10" s="3">
         <v>7.1590017415213195E-4</v>
       </c>
-      <c r="E6" s="4">
+      <c r="E10" s="3">
         <v>-2.71639045616228</v>
       </c>
-      <c r="F6" s="7">
+      <c r="F10" s="6">
         <v>9.3316692027003399E-3</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A7" s="3"/>
-      <c r="B7" s="4" t="s">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A11" s="7"/>
+      <c r="B11" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="C7" s="4">
+      <c r="C11" s="3">
         <v>-9.9780477580083495E-4</v>
       </c>
-      <c r="D7" s="4">
+      <c r="D11" s="3">
         <v>7.92584277725123E-4</v>
       </c>
-      <c r="E7" s="4">
+      <c r="E11" s="3">
         <v>-1.25892577463779</v>
       </c>
-      <c r="F7" s="4">
+      <c r="F11" s="3">
         <v>0.21454891644624999</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A8" s="3"/>
-      <c r="B8" s="4" t="s">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A12" s="7"/>
+      <c r="B12" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="C8" s="5">
+      <c r="C12" s="4">
         <v>8.3681496125827406E-5</v>
       </c>
-      <c r="D8" s="5">
+      <c r="D12" s="4">
         <v>6.26436959842307E-5</v>
       </c>
-      <c r="E8" s="4">
+      <c r="E12" s="3">
         <v>1.3358326773518101</v>
       </c>
-      <c r="F8" s="4">
+      <c r="F12" s="3">
         <v>0.188320928152656</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A9" s="3"/>
-      <c r="B9" s="4" t="s">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A13" s="7"/>
+      <c r="B13" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="C9" s="4">
+      <c r="C13" s="3">
         <v>-2.1651646073451799E-4</v>
       </c>
-      <c r="D9" s="4">
+      <c r="D13" s="3">
         <v>4.5990566625403001E-4</v>
       </c>
-      <c r="E9" s="4">
+      <c r="E13" s="3">
         <v>-0.47078450347886103</v>
       </c>
-      <c r="F9" s="4">
+      <c r="F13" s="3">
         <v>0.64006878265723399</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A10" s="3" t="s">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A14" s="8" t="s">
+        <v>15</v>
+      </c>
+      <c r="B14" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="C14" s="3">
+        <v>-9.5468806928554299E-4</v>
+      </c>
+      <c r="D14" s="3">
+        <v>3.4735442418317098E-4</v>
+      </c>
+      <c r="E14" s="3">
+        <v>-2.7484551881858401</v>
+      </c>
+      <c r="F14" s="6">
+        <v>8.5863891817765103E-3</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A15" s="9"/>
+      <c r="B15" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="C15" s="4">
+        <v>4.7400931557206599E-7</v>
+      </c>
+      <c r="D15" s="3">
+        <v>3.8456151478368102E-4</v>
+      </c>
+      <c r="E15" s="3">
+        <v>1.2325968599294201E-3</v>
+      </c>
+      <c r="F15" s="3">
+        <v>0.99902197837529505</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A16" s="9"/>
+      <c r="B16" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="C16" s="4">
+        <v>4.3181414524067597E-5</v>
+      </c>
+      <c r="D16" s="4">
+        <v>3.0394691512791901E-5</v>
+      </c>
+      <c r="E16" s="3">
+        <v>1.4206893498456601</v>
+      </c>
+      <c r="F16" s="3">
+        <v>0.162299507673272</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A17" s="10"/>
+      <c r="B17" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="C17" s="3">
+        <v>2.7412225349781997E-4</v>
+      </c>
+      <c r="D17" s="3">
+        <v>2.2314601064239801E-4</v>
+      </c>
+      <c r="E17" s="3">
+        <v>1.22844344251851</v>
+      </c>
+      <c r="F17" s="3">
+        <v>0.225666688292817</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A18" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="B10" s="7" t="s">
+      <c r="B18" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="C10" s="4">
+      <c r="C18" s="3">
         <v>1.4935788363256001E-3</v>
       </c>
-      <c r="D10" s="4">
+      <c r="D18" s="3">
         <v>5.8854471736806196E-4</v>
       </c>
-      <c r="E10" s="4">
+      <c r="E18" s="3">
         <v>2.53774911616707</v>
       </c>
-      <c r="F10" s="7">
+      <c r="F18" s="6">
         <v>1.4689736612161599E-2</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A11" s="3"/>
-      <c r="B11" s="4" t="s">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A19" s="7"/>
+      <c r="B19" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="C11" s="4">
+      <c r="C19" s="3">
         <v>1.1204974297703901E-3</v>
       </c>
-      <c r="D11" s="4">
+      <c r="D19" s="3">
         <v>6.5158705999277303E-4</v>
       </c>
-      <c r="E11" s="4">
+      <c r="E19" s="3">
         <v>1.7196434652689701</v>
       </c>
-      <c r="F11" s="4">
+      <c r="F19" s="3">
         <v>9.2369264111951205E-2</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A12" s="3"/>
-      <c r="B12" s="4" t="s">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A20" s="7"/>
+      <c r="B20" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="C12" s="5">
+      <c r="C20" s="4">
         <v>6.3284680573916897E-5</v>
       </c>
-      <c r="D12" s="5">
+      <c r="D20" s="4">
         <v>5.1499661096737001E-5</v>
       </c>
-      <c r="E12" s="4">
+      <c r="E20" s="3">
         <v>1.22883683554816</v>
       </c>
-      <c r="F12" s="4">
+      <c r="F20" s="3">
         <v>0.22552054751561801</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A13" s="3"/>
-      <c r="B13" s="7" t="s">
+    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A21" s="7"/>
+      <c r="B21" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="C13" s="4">
+      <c r="C21" s="3">
         <v>-8.3962398204233E-4</v>
       </c>
-      <c r="D13" s="4">
+      <c r="D21" s="3">
         <v>3.7809049380665202E-4</v>
       </c>
-      <c r="E13" s="4">
+      <c r="E21" s="3">
         <v>-2.2206958275753301</v>
       </c>
-      <c r="F13" s="7">
+      <c r="F21" s="6">
         <v>3.1449266952414602E-2</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A14" s="3" t="s">
+    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A22" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="B22" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="C22" s="3">
+        <v>7.5276848576755098E-4</v>
+      </c>
+      <c r="D22" s="3">
+        <v>3.10765531586891E-4</v>
+      </c>
+      <c r="E22" s="3">
+        <v>2.4223036638703701</v>
+      </c>
+      <c r="F22" s="6">
+        <v>1.95122412343436E-2</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A23" s="9"/>
+      <c r="B23" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="C23" s="3">
+        <v>2.0544563999823199E-4</v>
+      </c>
+      <c r="D23" s="3">
+        <v>3.44053379629879E-4</v>
+      </c>
+      <c r="E23" s="3">
+        <v>0.59713303853966804</v>
+      </c>
+      <c r="F23" s="3">
+        <v>0.55341140299014202</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A24" s="9"/>
+      <c r="B24" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="C24" s="4">
+        <v>5.8567293354296502E-6</v>
+      </c>
+      <c r="D24" s="4">
+        <v>2.7193039177792001E-5</v>
+      </c>
+      <c r="E24" s="3">
+        <v>0.215376048890214</v>
+      </c>
+      <c r="F24" s="3">
+        <v>0.83044734359580896</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A25" s="10"/>
+      <c r="B25" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="C25" s="4">
+        <v>-9.0730183629321296E-5</v>
+      </c>
+      <c r="D25" s="3">
+        <v>1.9964072368403301E-4</v>
+      </c>
+      <c r="E25" s="3">
+        <v>-0.45446731485965702</v>
+      </c>
+      <c r="F25" s="3">
+        <v>0.65167723877834804</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A26" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="B14" s="4" t="s">
+      <c r="B26" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="C14" s="4">
+      <c r="C26" s="3">
         <v>-2.7023531069502501E-4</v>
       </c>
-      <c r="D14" s="4">
+      <c r="D26" s="3">
         <v>3.7537791242540903E-4</v>
       </c>
-      <c r="E14" s="4">
+      <c r="E26" s="3">
         <v>-0.71990200208895705</v>
       </c>
-      <c r="F14" s="4">
+      <c r="F26" s="3">
         <v>0.47530801633141301</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A15" s="3"/>
-      <c r="B15" s="4" t="s">
+    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A27" s="7"/>
+      <c r="B27" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="C15" s="4">
+      <c r="C27" s="3">
         <v>-1.6023596752714399E-4</v>
       </c>
-      <c r="D15" s="4">
+      <c r="D27" s="3">
         <v>4.1558675683522499E-4</v>
       </c>
-      <c r="E15" s="4">
+      <c r="E27" s="3">
         <v>-0.38556562472628397</v>
       </c>
-      <c r="F15" s="4">
+      <c r="F27" s="3">
         <v>0.70163509696710702</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A16" s="3"/>
-      <c r="B16" s="7" t="s">
+    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A28" s="7"/>
+      <c r="B28" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="C16" s="5">
+      <c r="C28" s="4">
         <v>9.2965474620186606E-5</v>
       </c>
-      <c r="D16" s="5">
+      <c r="D28" s="4">
         <v>3.2846841884096897E-5</v>
       </c>
-      <c r="E16" s="4">
+      <c r="E28" s="3">
         <v>2.8302713225284801</v>
       </c>
-      <c r="F16" s="7">
+      <c r="F28" s="6">
         <v>6.9268179950745896E-3</v>
       </c>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A17" s="3"/>
-      <c r="B17" s="7" t="s">
+    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A29" s="7"/>
+      <c r="B29" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="C17" s="4">
+      <c r="C29" s="3">
         <v>-5.5677644615110904E-4</v>
       </c>
-      <c r="D17" s="4">
+      <c r="D29" s="3">
         <v>2.41148745515416E-4</v>
       </c>
-      <c r="E17" s="4">
+      <c r="E29" s="3">
         <v>-2.3088506845063201</v>
       </c>
-      <c r="F17" s="7">
+      <c r="F29" s="6">
         <v>2.5600307321182601E-2</v>
       </c>
     </row>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A30" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="B30" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="C30" s="3">
+        <v>7.5276848576755098E-4</v>
+      </c>
+      <c r="D30" s="3">
+        <v>3.10765531586891E-4</v>
+      </c>
+      <c r="E30" s="3">
+        <v>2.4223036638703701</v>
+      </c>
+      <c r="F30" s="6">
+        <v>1.95122412343436E-2</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A31" s="9"/>
+      <c r="B31" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="C31" s="3">
+        <v>2.0544563999823199E-4</v>
+      </c>
+      <c r="D31" s="3">
+        <v>3.44053379629879E-4</v>
+      </c>
+      <c r="E31" s="3">
+        <v>0.59713303853966804</v>
+      </c>
+      <c r="F31" s="3">
+        <v>0.55341140299014202</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A32" s="9"/>
+      <c r="B32" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="C32" s="4">
+        <v>5.8567293354296502E-6</v>
+      </c>
+      <c r="D32" s="4">
+        <v>2.7193039177792001E-5</v>
+      </c>
+      <c r="E32" s="3">
+        <v>0.215376048890214</v>
+      </c>
+      <c r="F32" s="3">
+        <v>0.83044734359580896</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A33" s="10"/>
+      <c r="B33" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="C33" s="4">
+        <v>-9.0730183629321296E-5</v>
+      </c>
+      <c r="D33" s="3">
+        <v>1.9964072368403301E-4</v>
+      </c>
+      <c r="E33" s="3">
+        <v>-0.45446731485965702</v>
+      </c>
+      <c r="F33" s="3">
+        <v>0.65167723877834804</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A34" s="8" t="s">
+        <v>17</v>
+      </c>
+      <c r="B34" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="C34" s="3">
+        <v>4.7050750518333299E-4</v>
+      </c>
+      <c r="D34" s="3">
+        <v>2.3595991593848599E-4</v>
+      </c>
+      <c r="E34" s="3">
+        <v>1.9940145482421401</v>
+      </c>
+      <c r="F34" s="5">
+        <v>5.2231351194580097E-2</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A35" s="9"/>
+      <c r="B35" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="C35" s="3">
+        <v>-3.3672767016649499E-4</v>
+      </c>
+      <c r="D35" s="3">
+        <v>2.61234912769337E-4</v>
+      </c>
+      <c r="E35" s="3">
+        <v>-1.2889841813135301</v>
+      </c>
+      <c r="F35" s="3">
+        <v>0.20399058107860699</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A36" s="9"/>
+      <c r="B36" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="C36" s="4">
+        <v>-1.4054752388213601E-5</v>
+      </c>
+      <c r="D36" s="4">
+        <v>2.0647293815819101E-5</v>
+      </c>
+      <c r="E36" s="3">
+        <v>-0.68070675574178297</v>
+      </c>
+      <c r="F36" s="3">
+        <v>0.499544802222599</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A37" s="10"/>
+      <c r="B37" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="C37" s="3">
+        <v>-1.6175952732976799E-4</v>
+      </c>
+      <c r="D37" s="3">
+        <v>1.51584405573665E-4</v>
+      </c>
+      <c r="E37" s="3">
+        <v>-1.0671251222551299</v>
+      </c>
+      <c r="F37" s="3">
+        <v>0.29160706442622902</v>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="4">
+  <mergeCells count="9">
+    <mergeCell ref="A26:A29"/>
+    <mergeCell ref="A18:A21"/>
+    <mergeCell ref="A10:A13"/>
+    <mergeCell ref="A2:A5"/>
+    <mergeCell ref="A34:A37"/>
+    <mergeCell ref="A30:A33"/>
     <mergeCell ref="A14:A17"/>
-    <mergeCell ref="A10:A13"/>
     <mergeCell ref="A6:A9"/>
-    <mergeCell ref="A2:A5"/>
+    <mergeCell ref="A22:A25"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -763,7 +1196,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F17"/>
+  <dimension ref="A1:F33"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="15.28515625" bestFit="1" customWidth="1"/>
@@ -790,307 +1223,607 @@
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A2" s="3" t="s">
+      <c r="A2" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="B2" s="4" t="s">
+      <c r="B2" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="C2" s="5">
+      <c r="C2" s="4">
         <v>8.8737323696130597E-5</v>
       </c>
-      <c r="D2" s="4">
+      <c r="D2" s="3">
         <v>1.4333539470505301E-4</v>
       </c>
-      <c r="E2" s="4">
+      <c r="E2" s="3">
         <v>0.619088703657104</v>
       </c>
-      <c r="F2" s="4">
+      <c r="F2" s="3">
         <v>0.53920168256468504</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A3" s="3"/>
-      <c r="B3" s="4" t="s">
+      <c r="A3" s="7"/>
+      <c r="B3" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="C3" s="4">
+      <c r="C3" s="3">
         <v>-3.5638036387647799E-4</v>
       </c>
-      <c r="D3" s="4">
+      <c r="D3" s="3">
         <v>3.0386801340194302E-4</v>
       </c>
-      <c r="E3" s="4">
+      <c r="E3" s="3">
         <v>-1.1728130245978701</v>
       </c>
-      <c r="F3" s="4">
+      <c r="F3" s="3">
         <v>0.24747980038165601</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A4" s="3"/>
-      <c r="B4" s="7" t="s">
+      <c r="A4" s="7"/>
+      <c r="B4" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="C4" s="5">
+      <c r="C4" s="4">
         <v>-9.3952787693282695E-5</v>
       </c>
-      <c r="D4" s="5">
+      <c r="D4" s="4">
         <v>4.6540090692536602E-5</v>
       </c>
-      <c r="E4" s="4">
+      <c r="E4" s="3">
         <v>-2.0187495618342099</v>
       </c>
-      <c r="F4" s="7">
+      <c r="F4" s="6">
         <v>4.99276235621448E-2</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A5" s="3"/>
-      <c r="B5" s="4" t="s">
+      <c r="A5" s="7"/>
+      <c r="B5" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="C5" s="5">
+      <c r="C5" s="4">
         <v>-5.1790506761720298E-5</v>
       </c>
-      <c r="D5" s="4">
+      <c r="D5" s="3">
         <v>2.1520893950268801E-4</v>
       </c>
-      <c r="E5" s="4">
+      <c r="E5" s="3">
         <v>-0.24065220934316001</v>
       </c>
-      <c r="F5" s="4">
+      <c r="F5" s="3">
         <v>0.81099554817921404</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A6" s="3" t="s">
+      <c r="A6" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="B6" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="C6" s="3">
+        <v>2.5130292757481E-4</v>
+      </c>
+      <c r="D6" s="4">
+        <v>8.3464775240331795E-5</v>
+      </c>
+      <c r="E6" s="3">
+        <v>3.0108860516451199</v>
+      </c>
+      <c r="F6" s="6">
+        <v>4.3952204536846602E-3</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A7" s="7"/>
+      <c r="B7" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="C7" s="3">
+        <v>-1.6254749312297599E-4</v>
+      </c>
+      <c r="D7" s="3">
+        <v>1.76943562987414E-4</v>
+      </c>
+      <c r="E7" s="3">
+        <v>-0.91864033016300495</v>
+      </c>
+      <c r="F7" s="3">
+        <v>0.36352953240204899</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A8" s="7"/>
+      <c r="B8" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="C8" s="4">
+        <v>-4.0690371551118497E-5</v>
+      </c>
+      <c r="D8" s="4">
+        <v>2.7100481477798499E-5</v>
+      </c>
+      <c r="E8" s="3">
+        <v>-1.50146304907731</v>
+      </c>
+      <c r="F8" s="3">
+        <v>0.14071724489836901</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A9" s="7"/>
+      <c r="B9" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="C9" s="4">
+        <v>-2.2433702309757401E-5</v>
+      </c>
+      <c r="D9" s="3">
+        <v>1.2531702865341699E-4</v>
+      </c>
+      <c r="E9" s="3">
+        <v>-0.17901559389666899</v>
+      </c>
+      <c r="F9" s="3">
+        <v>0.85878625382581697</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A10" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="B6" s="4" t="s">
+      <c r="B10" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="C6" s="5">
+      <c r="C10" s="4">
         <v>5.3835873445009803E-5</v>
       </c>
-      <c r="D6" s="4">
+      <c r="D10" s="3">
         <v>1.05802027861303E-4</v>
       </c>
-      <c r="E6" s="4">
+      <c r="E10" s="3">
         <v>0.50883593191222998</v>
       </c>
-      <c r="F6" s="4">
+      <c r="F10" s="3">
         <v>0.61353001426340603</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A7" s="3"/>
-      <c r="B7" s="4" t="s">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A11" s="7"/>
+      <c r="B11" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="C7" s="4">
+      <c r="C11" s="3">
         <v>-3.8980255679120398E-4</v>
       </c>
-      <c r="D7" s="4">
+      <c r="D11" s="3">
         <v>2.24298067384314E-4</v>
       </c>
-      <c r="E7" s="4">
+      <c r="E11" s="3">
         <v>-1.7378774651825799</v>
       </c>
-      <c r="F7" s="4">
+      <c r="F11" s="3">
         <v>8.9560493894961901E-2</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A8" s="3"/>
-      <c r="B8" s="4" t="s">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A12" s="7"/>
+      <c r="B12" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="C8" s="5">
+      <c r="C12" s="4">
         <v>-2.8143767760553299E-5</v>
       </c>
-      <c r="D8" s="5">
+      <c r="D12" s="4">
         <v>3.4353245283565202E-5</v>
       </c>
-      <c r="E8" s="4">
+      <c r="E12" s="3">
         <v>-0.81924626125548095</v>
       </c>
-      <c r="F8" s="4">
+      <c r="F12" s="3">
         <v>0.417270597697602</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A9" s="3"/>
-      <c r="B9" s="4" t="s">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A13" s="7"/>
+      <c r="B13" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="C9" s="5">
+      <c r="C13" s="4">
         <v>-6.7848175045799597E-5</v>
       </c>
-      <c r="D9" s="4">
+      <c r="D13" s="3">
         <v>1.5885498665642699E-4</v>
       </c>
-      <c r="E9" s="4">
+      <c r="E13" s="3">
         <v>-0.42710761855113999</v>
       </c>
-      <c r="F9" s="4">
+      <c r="F13" s="3">
         <v>0.67148261224119599</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A10" s="3" t="s">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A14" s="7" t="s">
+        <v>15</v>
+      </c>
+      <c r="B14" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="C14" s="3">
+        <v>2.4428145382339298E-4</v>
+      </c>
+      <c r="D14" s="4">
+        <v>6.2616360428445402E-5</v>
+      </c>
+      <c r="E14" s="3">
+        <v>3.9012400617334499</v>
+      </c>
+      <c r="F14" s="6">
+        <v>3.39672493895188E-4</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A15" s="7"/>
+      <c r="B15" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="C15" s="3">
+        <v>-2.0654003846089201E-4</v>
+      </c>
+      <c r="D15" s="3">
+        <v>1.3274536334172501E-4</v>
+      </c>
+      <c r="E15" s="3">
+        <v>-1.55591150802909</v>
+      </c>
+      <c r="F15" s="3">
+        <v>0.12723318591701499</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A16" s="7"/>
+      <c r="B16" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="C16" s="4">
+        <v>-1.58699129583369E-5</v>
+      </c>
+      <c r="D16" s="4">
+        <v>2.0331133835944801E-5</v>
+      </c>
+      <c r="E16" s="3">
+        <v>-0.78057195857318196</v>
+      </c>
+      <c r="F16" s="3">
+        <v>0.43943166741512302</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A17" s="7"/>
+      <c r="B17" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="C17" s="4">
+        <v>6.48853101011375E-6</v>
+      </c>
+      <c r="D17" s="4">
+        <v>9.4014465520209401E-5</v>
+      </c>
+      <c r="E17" s="3">
+        <v>6.90163048229952E-2</v>
+      </c>
+      <c r="F17" s="3">
+        <v>0.94530418917923997</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A18" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="B10" s="4" t="s">
+      <c r="B18" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="C10" s="4">
+      <c r="C18" s="3">
         <v>1.46424350741536E-4</v>
       </c>
-      <c r="D10" s="4">
+      <c r="D18" s="3">
         <v>1.05933110579384E-4</v>
       </c>
-      <c r="E10" s="4">
+      <c r="E18" s="3">
         <v>1.3822340337283801</v>
       </c>
-      <c r="F10" s="4">
+      <c r="F18" s="3">
         <v>0.17420695554378601</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A11" s="3"/>
-      <c r="B11" s="4" t="s">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A19" s="7"/>
+      <c r="B19" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="C11" s="4">
+      <c r="C19" s="3">
         <v>3.86325328396926E-4</v>
       </c>
-      <c r="D11" s="4">
+      <c r="D19" s="3">
         <v>2.24575959981718E-4</v>
       </c>
-      <c r="E11" s="4">
+      <c r="E19" s="3">
         <v>1.7202434687505099</v>
       </c>
-      <c r="F11" s="4">
+      <c r="F19" s="3">
         <v>9.2749498762672397E-2</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A12" s="3"/>
-      <c r="B12" s="7" t="s">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A20" s="7"/>
+      <c r="B20" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="C12" s="5">
+      <c r="C20" s="4">
         <v>7.9444135783364797E-5</v>
       </c>
-      <c r="D12" s="5">
+      <c r="D20" s="4">
         <v>3.4395807008115198E-5</v>
       </c>
-      <c r="E12" s="4">
+      <c r="E20" s="3">
         <v>2.3097040800531601</v>
       </c>
-      <c r="F12" s="7">
+      <c r="F20" s="6">
         <v>2.5890658437057599E-2</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A13" s="3"/>
-      <c r="B13" s="4" t="s">
+    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A21" s="7"/>
+      <c r="B21" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="C13" s="4">
+      <c r="C21" s="3">
         <v>-1.5823880287253001E-4</v>
       </c>
-      <c r="D13" s="4">
+      <c r="D21" s="3">
         <v>1.59051798984626E-4</v>
       </c>
-      <c r="E13" s="4">
+      <c r="E21" s="3">
         <v>-0.994888482134209</v>
       </c>
-      <c r="F13" s="4">
+      <c r="F21" s="3">
         <v>0.32548805260610297</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A14" s="3" t="s">
+    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A22" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="B22" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="C22" s="4">
+        <v>-3.3644858381696802E-5</v>
+      </c>
+      <c r="D22" s="4">
+        <v>6.1976488364197705E-5</v>
+      </c>
+      <c r="E22" s="3">
+        <v>-0.54286487133615402</v>
+      </c>
+      <c r="F22" s="3">
+        <v>0.59009230469615304</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A23" s="7"/>
+      <c r="B23" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="C23" s="4">
+        <v>8.2676407847088193E-5</v>
+      </c>
+      <c r="D23" s="3">
+        <v>1.3138884806233799E-4</v>
+      </c>
+      <c r="E23" s="3">
+        <v>0.62924981127669399</v>
+      </c>
+      <c r="F23" s="3">
+        <v>0.53259349499761299</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A24" s="7"/>
+      <c r="B24" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="C24" s="4">
+        <v>5.9204307406862699E-5</v>
+      </c>
+      <c r="D24" s="4">
+        <v>2.0123371447855002E-5</v>
+      </c>
+      <c r="E24" s="3">
+        <v>2.9420670169646601</v>
+      </c>
+      <c r="F24" s="6">
+        <v>5.2873646755308996E-3</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A25" s="7"/>
+      <c r="B25" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="C25" s="4">
+        <v>-7.24354736861226E-5</v>
+      </c>
+      <c r="D25" s="4">
+        <v>9.3053738488009695E-5</v>
+      </c>
+      <c r="E25" s="3">
+        <v>-0.77842626060054698</v>
+      </c>
+      <c r="F25" s="3">
+        <v>0.44068137194206702</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A26" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="B14" s="4" t="s">
+      <c r="B26" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="C14" s="5">
+      <c r="C26" s="4">
         <v>5.7102313957604099E-5</v>
       </c>
-      <c r="D14" s="4">
+      <c r="D26" s="3">
         <v>1.0228784914160101E-4</v>
       </c>
-      <c r="E14" s="4">
+      <c r="E26" s="3">
         <v>0.55825119441660298</v>
       </c>
-      <c r="F14" s="4">
+      <c r="F26" s="3">
         <v>0.57963688266824898</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A15" s="3"/>
-      <c r="B15" s="4" t="s">
+    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A27" s="7"/>
+      <c r="B27" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="C15" s="4">
+      <c r="C27" s="3">
         <v>1.5262466026198199E-4</v>
       </c>
-      <c r="D15" s="4">
+      <c r="D27" s="3">
         <v>2.1684808262309999E-4</v>
       </c>
-      <c r="E15" s="4">
+      <c r="E27" s="3">
         <v>0.70383218710425999</v>
       </c>
-      <c r="F15" s="4">
+      <c r="F27" s="3">
         <v>0.48542133735885001</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A16" s="3"/>
-      <c r="B16" s="7" t="s">
+    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A28" s="7"/>
+      <c r="B28" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="C16" s="5">
+      <c r="C28" s="4">
         <v>7.3351506781873705E-5</v>
       </c>
-      <c r="D16" s="5">
+      <c r="D28" s="4">
         <v>3.3212213812160298E-5</v>
       </c>
-      <c r="E16" s="4">
+      <c r="E28" s="3">
         <v>2.2085702325274301</v>
       </c>
-      <c r="F16" s="7">
+      <c r="F28" s="6">
         <v>3.2715345058187399E-2</v>
       </c>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A17" s="3"/>
-      <c r="B17" s="4" t="s">
+    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A29" s="7"/>
+      <c r="B29" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="C17" s="5">
+      <c r="C29" s="4">
         <v>-7.2515487086999606E-5</v>
       </c>
-      <c r="D17" s="4">
+      <c r="D29" s="3">
         <v>1.53578671779378E-4</v>
       </c>
-      <c r="E17" s="4">
+      <c r="E29" s="3">
         <v>-0.47217159939481201</v>
       </c>
-      <c r="F17" s="4">
+      <c r="F29" s="3">
         <v>0.63924847561166498</v>
       </c>
     </row>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A30" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="B30" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="C30" s="4">
+        <v>-1.6578921541507301E-5</v>
+      </c>
+      <c r="D30" s="4">
+        <v>6.5151308724298106E-5</v>
+      </c>
+      <c r="E30" s="3">
+        <v>-0.25446797410723598</v>
+      </c>
+      <c r="F30" s="3">
+        <v>0.80037585825981605</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A31" s="7"/>
+      <c r="B31" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="C31" s="4">
+        <v>-1.06621082374178E-6</v>
+      </c>
+      <c r="D31" s="3">
+        <v>1.3811940025928001E-4</v>
+      </c>
+      <c r="E31" s="3">
+        <v>-7.7194863410952599E-3</v>
+      </c>
+      <c r="F31" s="3">
+        <v>0.99387735320458503</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A32" s="7"/>
+      <c r="B32" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="C32" s="4">
+        <v>6.5520189952899299E-5</v>
+      </c>
+      <c r="D32" s="4">
+        <v>2.11542154190572E-5</v>
+      </c>
+      <c r="E32" s="3">
+        <v>3.0972640041225099</v>
+      </c>
+      <c r="F32" s="6">
+        <v>3.4749304931421302E-3</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A33" s="7"/>
+      <c r="B33" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="C33" s="4">
+        <v>-6.5209017198555506E-5</v>
+      </c>
+      <c r="D33" s="4">
+        <v>9.7820528464865694E-5</v>
+      </c>
+      <c r="E33" s="3">
+        <v>-0.66661894207591299</v>
+      </c>
+      <c r="F33" s="3">
+        <v>0.50866120136667603</v>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="4">
+  <mergeCells count="8">
+    <mergeCell ref="A26:A29"/>
+    <mergeCell ref="A18:A21"/>
+    <mergeCell ref="A10:A13"/>
+    <mergeCell ref="A2:A5"/>
+    <mergeCell ref="A30:A33"/>
+    <mergeCell ref="A22:A25"/>
     <mergeCell ref="A14:A17"/>
-    <mergeCell ref="A10:A13"/>
     <mergeCell ref="A6:A9"/>
-    <mergeCell ref="A2:A5"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>